<commit_message>
forecast prep + haver pull (May)
</commit_message>
<xml_diff>
--- a/data/monthly_state_ui.xlsx
+++ b/data/monthly_state_ui.xlsx
@@ -355,7 +355,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:R664"/>
+  <dimension ref="A1:R665"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="20.7109375" style="2" customWidth="1"/>
@@ -35576,7 +35576,7 @@
         <v>15053</v>
       </c>
       <c r="R662">
-        <v>470274</v>
+        <v>471070</v>
       </c>
     </row>
     <row r="663">
@@ -35626,13 +35626,13 @@
         <v>2054381</v>
       </c>
       <c r="P663">
-        <v>5520</v>
+        <v>5514</v>
       </c>
       <c r="Q663">
-        <v>15069</v>
+        <v>15071</v>
       </c>
       <c r="R663">
-        <v>472115</v>
+        <v>472141</v>
       </c>
     </row>
     <row r="664">
@@ -35682,10 +35682,24 @@
         <v>2078927</v>
       </c>
       <c r="P664">
-        <v>5526</v>
+        <v>5516</v>
       </c>
       <c r="Q664">
-        <v>15086</v>
+        <v>15088</v>
+      </c>
+      <c r="R664">
+        <v>471183</v>
+      </c>
+    </row>
+    <row r="665">
+      <c r="A665" s="2">
+        <v>45777</v>
+      </c>
+      <c r="P665">
+        <v>5522</v>
+      </c>
+      <c r="Q665">
+        <v>15101</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
haver pull (June FIM)
</commit_message>
<xml_diff>
--- a/data/monthly_state_ui.xlsx
+++ b/data/monthly_state_ui.xlsx
@@ -355,7 +355,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:R665"/>
+  <dimension ref="A1:R666"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="20.7109375" style="2" customWidth="1"/>
@@ -35632,7 +35632,7 @@
         <v>15071</v>
       </c>
       <c r="R663">
-        <v>472141</v>
+        <v>474386</v>
       </c>
     </row>
     <row r="664">
@@ -35682,24 +35682,41 @@
         <v>2078927</v>
       </c>
       <c r="P664">
-        <v>5516</v>
+        <v>5515</v>
       </c>
       <c r="Q664">
-        <v>15088</v>
+        <v>15087</v>
       </c>
       <c r="R664">
-        <v>471183</v>
+        <v>474713</v>
       </c>
     </row>
     <row r="665">
       <c r="A665" s="2">
         <v>45777</v>
       </c>
+      <c r="C665">
+        <v>1877</v>
+      </c>
       <c r="P665">
-        <v>5522</v>
+        <v>5518</v>
       </c>
       <c r="Q665">
-        <v>15101</v>
+        <v>15098</v>
+      </c>
+      <c r="R665">
+        <v>475961</v>
+      </c>
+    </row>
+    <row r="666">
+      <c r="A666" s="2">
+        <v>45808</v>
+      </c>
+      <c r="P666">
+        <v>5518</v>
+      </c>
+      <c r="Q666">
+        <v>15119</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
edits to forecast sheet prep
</commit_message>
<xml_diff>
--- a/data/monthly_state_ui.xlsx
+++ b/data/monthly_state_ui.xlsx
@@ -35481,7 +35481,7 @@
         <v>541872</v>
       </c>
       <c r="E661">
-        <v>194341</v>
+        <v>194486</v>
       </c>
       <c r="F661">
         <v>9204452</v>
@@ -35496,7 +35496,7 @@
         <v>463.85</v>
       </c>
       <c r="J661">
-        <v>39.38</v>
+        <v>39.39</v>
       </c>
       <c r="K661">
         <v>15.27</v>
@@ -35511,7 +35511,7 @@
         <v>5333073</v>
       </c>
       <c r="O661">
-        <v>2050422</v>
+        <v>2050567</v>
       </c>
       <c r="P661">
         <v>5512</v>
@@ -35537,7 +35537,7 @@
         <v>689057</v>
       </c>
       <c r="E662">
-        <v>180879</v>
+        <v>181369</v>
       </c>
       <c r="F662">
         <v>9270888</v>
@@ -35552,7 +35552,7 @@
         <v>469.31</v>
       </c>
       <c r="J662">
-        <v>38.92</v>
+        <v>38.94</v>
       </c>
       <c r="K662">
         <v>15.17</v>
@@ -35567,7 +35567,7 @@
         <v>5341621</v>
       </c>
       <c r="O662">
-        <v>2046798</v>
+        <v>2047433</v>
       </c>
       <c r="P662">
         <v>5524</v>
@@ -35593,7 +35593,7 @@
         <v>483723</v>
       </c>
       <c r="E663">
-        <v>165056</v>
+        <v>165517</v>
       </c>
       <c r="F663">
         <v>8657563</v>
@@ -35608,7 +35608,7 @@
         <v>471.52</v>
       </c>
       <c r="J663">
-        <v>39.2</v>
+        <v>39.22</v>
       </c>
       <c r="K663">
         <v>15.21</v>
@@ -35623,7 +35623,7 @@
         <v>5334787</v>
       </c>
       <c r="O663">
-        <v>2054385</v>
+        <v>2055481</v>
       </c>
       <c r="P663">
         <v>5514</v>
@@ -35649,7 +35649,7 @@
         <v>431634</v>
       </c>
       <c r="E664">
-        <v>188320</v>
+        <v>188778</v>
       </c>
       <c r="F664">
         <v>9621697</v>
@@ -35664,7 +35664,7 @@
         <v>467.76</v>
       </c>
       <c r="J664">
-        <v>39.55</v>
+        <v>39.58</v>
       </c>
       <c r="K664">
         <v>15.3</v>
@@ -35679,7 +35679,7 @@
         <v>5357362</v>
       </c>
       <c r="O664">
-        <v>2078931</v>
+        <v>2080485</v>
       </c>
       <c r="P664">
         <v>5515</v>
@@ -35696,31 +35696,31 @@
         <v>45777</v>
       </c>
       <c r="B665">
-        <v>942880</v>
+        <v>942921</v>
       </c>
       <c r="C665">
         <v>1877</v>
       </c>
       <c r="D665">
-        <v>401311</v>
+        <v>401308</v>
       </c>
       <c r="E665">
-        <v>188757</v>
+        <v>189319</v>
       </c>
       <c r="F665">
-        <v>7912629</v>
+        <v>7912998</v>
       </c>
       <c r="G665">
-        <v>6972911</v>
+        <v>6972902</v>
       </c>
       <c r="H665">
-        <v>3204879</v>
+        <v>3204874</v>
       </c>
       <c r="I665">
         <v>468.53</v>
       </c>
       <c r="J665">
-        <v>39.43</v>
+        <v>39.47</v>
       </c>
       <c r="K665">
         <v>15.22</v>
@@ -35729,13 +35729,13 @@
         <v>458.19</v>
       </c>
       <c r="M665">
-        <v>36812035</v>
+        <v>36812030</v>
       </c>
       <c r="N665">
-        <v>5375536</v>
+        <v>5375533</v>
       </c>
       <c r="O665">
-        <v>2082073</v>
+        <v>2084189</v>
       </c>
       <c r="P665">
         <v>5526</v>
@@ -35761,10 +35761,10 @@
         <v>371539</v>
       </c>
       <c r="E666">
-        <v>173824</v>
+        <v>174208</v>
       </c>
       <c r="F666">
-        <v>7225007</v>
+        <v>7224989</v>
       </c>
       <c r="G666">
         <v>6139864</v>
@@ -35776,7 +35776,7 @@
         <v>465.28</v>
       </c>
       <c r="J666">
-        <v>39.71</v>
+        <v>39.76</v>
       </c>
       <c r="K666">
         <v>15.27</v>
@@ -35785,13 +35785,13 @@
         <v>458.9</v>
       </c>
       <c r="M666">
-        <v>36916439</v>
+        <v>36916434</v>
       </c>
       <c r="N666">
-        <v>5368103</v>
+        <v>5368100</v>
       </c>
       <c r="O666">
-        <v>2087387</v>
+        <v>2089887</v>
       </c>
       <c r="P666">
         <v>5515</v>
@@ -35808,46 +35808,46 @@
         <v>45838</v>
       </c>
       <c r="B667">
-        <v>1032107</v>
+        <v>1032546</v>
       </c>
       <c r="C667">
-        <v>1479.3</v>
+        <v>1860.9</v>
       </c>
       <c r="D667">
-        <v>460026</v>
+        <v>457397</v>
       </c>
       <c r="E667">
-        <v>180267</v>
+        <v>178940</v>
       </c>
       <c r="F667">
-        <v>8502534</v>
+        <v>8573393</v>
       </c>
       <c r="G667">
-        <v>6959332</v>
+        <v>6954177</v>
       </c>
       <c r="H667">
-        <v>3111116</v>
+        <v>3103168</v>
       </c>
       <c r="I667">
-        <v>455.85</v>
+        <v>455.59</v>
       </c>
       <c r="J667">
-        <v>39.53</v>
+        <v>39.55</v>
       </c>
       <c r="K667">
-        <v>15.29</v>
+        <v>15.3</v>
       </c>
       <c r="L667">
-        <v>459.72</v>
+        <v>459.7</v>
       </c>
       <c r="M667">
-        <v>37404150</v>
+        <v>37396197</v>
       </c>
       <c r="N667">
-        <v>5422572</v>
+        <v>5419940</v>
       </c>
       <c r="O667">
-        <v>2108100</v>
+        <v>2109273</v>
       </c>
       <c r="P667">
         <v>5525</v>
@@ -35863,32 +35863,47 @@
       <c r="A668" s="2">
         <v>45869</v>
       </c>
+      <c r="B668">
+        <v>985989</v>
+      </c>
+      <c r="C668">
+        <v>2004.2</v>
+      </c>
       <c r="D668">
-        <v>7515</v>
+        <v>508090</v>
       </c>
       <c r="E668">
-        <v>1472</v>
+        <v>182815</v>
+      </c>
+      <c r="F668">
+        <v>8405033</v>
+      </c>
+      <c r="G668">
+        <v>7256308</v>
       </c>
       <c r="H668">
-        <v>18748</v>
+        <v>3266414</v>
+      </c>
+      <c r="I668">
+        <v>458.42</v>
       </c>
       <c r="J668">
-        <v>36.09</v>
+        <v>39.51</v>
       </c>
       <c r="K668">
-        <v>15.41</v>
+        <v>15.32</v>
       </c>
       <c r="L668">
-        <v>461.53</v>
+        <v>461.49</v>
       </c>
       <c r="M668">
-        <v>34258073</v>
+        <v>37497786</v>
       </c>
       <c r="N668">
-        <v>4907961</v>
+        <v>5405904</v>
       </c>
       <c r="O668">
-        <v>1927742</v>
+        <v>2110258</v>
       </c>
       <c r="P668">
         <v>5530</v>

</xml_diff>

<commit_message>
pulling in Q4 data + December MPI
</commit_message>
<xml_diff>
--- a/data/monthly_state_ui.xlsx
+++ b/data/monthly_state_ui.xlsx
@@ -355,7 +355,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:R673"/>
+  <dimension ref="A1:R674"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="20.7109375" style="2" customWidth="1"/>
@@ -32882,10 +32882,10 @@
         <v>12105826</v>
       </c>
       <c r="P614">
-        <v>5150</v>
+        <v>5142</v>
       </c>
       <c r="Q614">
-        <v>13743</v>
+        <v>13715</v>
       </c>
       <c r="R614">
         <v>342295</v>
@@ -32938,10 +32938,10 @@
         <v>12600385</v>
       </c>
       <c r="P615">
-        <v>5154</v>
+        <v>5153</v>
       </c>
       <c r="Q615">
-        <v>13728</v>
+        <v>13718</v>
       </c>
       <c r="R615">
         <v>334159</v>
@@ -32994,10 +32994,10 @@
         <v>13044263</v>
       </c>
       <c r="P616">
-        <v>5192</v>
+        <v>5186</v>
       </c>
       <c r="Q616">
-        <v>13779</v>
+        <v>13773</v>
       </c>
       <c r="R616">
         <v>337880</v>
@@ -33050,10 +33050,10 @@
         <v>13246975</v>
       </c>
       <c r="P617">
-        <v>5187</v>
+        <v>5180</v>
       </c>
       <c r="Q617">
-        <v>13827</v>
+        <v>13819</v>
       </c>
       <c r="R617">
         <v>336247</v>
@@ -33106,10 +33106,10 @@
         <v>13354228</v>
       </c>
       <c r="P618">
-        <v>5174</v>
+        <v>5178</v>
       </c>
       <c r="Q618">
-        <v>13849</v>
+        <v>13865</v>
       </c>
       <c r="R618">
         <v>337543</v>
@@ -33162,10 +33162,10 @@
         <v>13081161</v>
       </c>
       <c r="P619">
-        <v>5199</v>
+        <v>5197</v>
       </c>
       <c r="Q619">
-        <v>13917</v>
+        <v>13947</v>
       </c>
       <c r="R619">
         <v>329898</v>
@@ -33218,10 +33218,10 @@
         <v>12415951</v>
       </c>
       <c r="P620">
-        <v>5177</v>
+        <v>5180</v>
       </c>
       <c r="Q620">
-        <v>13990</v>
+        <v>13967</v>
       </c>
       <c r="R620">
         <v>330467</v>
@@ -33274,10 +33274,10 @@
         <v>11621754</v>
       </c>
       <c r="P621">
-        <v>5155</v>
+        <v>5153</v>
       </c>
       <c r="Q621">
-        <v>14057</v>
+        <v>14095</v>
       </c>
       <c r="R621">
         <v>332900</v>
@@ -33330,10 +33330,10 @@
         <v>8844628</v>
       </c>
       <c r="P622">
-        <v>5139</v>
+        <v>5137</v>
       </c>
       <c r="Q622">
-        <v>14055</v>
+        <v>14078</v>
       </c>
       <c r="R622">
         <v>327369</v>
@@ -33389,7 +33389,7 @@
         <v>5132</v>
       </c>
       <c r="Q623">
-        <v>14035</v>
+        <v>14017</v>
       </c>
       <c r="R623">
         <v>324962</v>
@@ -33442,10 +33442,10 @@
         <v>5597412</v>
       </c>
       <c r="P624">
-        <v>5121</v>
+        <v>5124</v>
       </c>
       <c r="Q624">
-        <v>14035</v>
+        <v>14033</v>
       </c>
       <c r="R624">
         <v>331225</v>
@@ -33498,10 +33498,10 @@
         <v>4737809</v>
       </c>
       <c r="P625">
-        <v>5122</v>
+        <v>5121</v>
       </c>
       <c r="Q625">
-        <v>14071</v>
+        <v>14059</v>
       </c>
       <c r="R625">
         <v>332079</v>
@@ -33554,10 +33554,10 @@
         <v>4093576</v>
       </c>
       <c r="P626">
-        <v>5087</v>
+        <v>5089</v>
       </c>
       <c r="Q626">
-        <v>14091</v>
+        <v>14081</v>
       </c>
       <c r="R626">
         <v>335367</v>
@@ -33610,10 +33610,10 @@
         <v>3599436</v>
       </c>
       <c r="P627">
-        <v>5070</v>
+        <v>5069</v>
       </c>
       <c r="Q627">
-        <v>14097</v>
+        <v>14089</v>
       </c>
       <c r="R627">
         <v>339940</v>
@@ -33666,10 +33666,10 @@
         <v>3159034</v>
       </c>
       <c r="P628">
-        <v>5057</v>
+        <v>5052</v>
       </c>
       <c r="Q628">
-        <v>14116</v>
+        <v>14114</v>
       </c>
       <c r="R628">
         <v>343309</v>
@@ -33722,10 +33722,10 @@
         <v>2875535</v>
       </c>
       <c r="P629">
-        <v>5075</v>
+        <v>5068</v>
       </c>
       <c r="Q629">
-        <v>14137</v>
+        <v>14135</v>
       </c>
       <c r="R629">
         <v>349983</v>
@@ -33778,10 +33778,10 @@
         <v>2630865</v>
       </c>
       <c r="P630">
-        <v>5095</v>
+        <v>5100</v>
       </c>
       <c r="Q630">
-        <v>14145</v>
+        <v>14163</v>
       </c>
       <c r="R630">
         <v>342679</v>
@@ -33834,10 +33834,10 @@
         <v>2404027</v>
       </c>
       <c r="P631">
-        <v>5104</v>
+        <v>5107</v>
       </c>
       <c r="Q631">
-        <v>14168</v>
+        <v>14182</v>
       </c>
       <c r="R631">
         <v>349662</v>
@@ -33890,10 +33890,10 @@
         <v>2232756</v>
       </c>
       <c r="P632">
-        <v>5140</v>
+        <v>5137</v>
       </c>
       <c r="Q632">
-        <v>14280</v>
+        <v>14307</v>
       </c>
       <c r="R632">
         <v>357378</v>
@@ -33946,10 +33946,10 @@
         <v>2077763</v>
       </c>
       <c r="P633">
-        <v>5146</v>
+        <v>5144</v>
       </c>
       <c r="Q633">
-        <v>14264</v>
+        <v>14301</v>
       </c>
       <c r="R633">
         <v>362881</v>
@@ -34002,10 +34002,10 @@
         <v>1874576</v>
       </c>
       <c r="P634">
-        <v>5148</v>
+        <v>5149</v>
       </c>
       <c r="Q634">
-        <v>14269</v>
+        <v>14283</v>
       </c>
       <c r="R634">
         <v>366384</v>
@@ -34058,10 +34058,10 @@
         <v>1683174</v>
       </c>
       <c r="P635">
-        <v>5139</v>
+        <v>5140</v>
       </c>
       <c r="Q635">
-        <v>14301</v>
+        <v>14283</v>
       </c>
       <c r="R635">
         <v>365642</v>
@@ -34114,10 +34114,10 @@
         <v>1584506</v>
       </c>
       <c r="P636">
-        <v>5162</v>
+        <v>5163</v>
       </c>
       <c r="Q636">
-        <v>14337</v>
+        <v>14339</v>
       </c>
       <c r="R636">
         <v>366244</v>
@@ -34170,10 +34170,10 @@
         <v>1517217</v>
       </c>
       <c r="P637">
-        <v>5136</v>
+        <v>5133</v>
       </c>
       <c r="Q637">
-        <v>14364</v>
+        <v>14358</v>
       </c>
       <c r="R637">
         <v>373987</v>
@@ -34229,7 +34229,7 @@
         <v>5199</v>
       </c>
       <c r="Q638">
-        <v>14411</v>
+        <v>14405</v>
       </c>
       <c r="R638">
         <v>379392</v>
@@ -34282,10 +34282,10 @@
         <v>1459580</v>
       </c>
       <c r="P639">
-        <v>5219</v>
+        <v>5218</v>
       </c>
       <c r="Q639">
-        <v>14439</v>
+        <v>14433</v>
       </c>
       <c r="R639">
         <v>387843</v>
@@ -34338,10 +34338,10 @@
         <v>1421645</v>
       </c>
       <c r="P640">
-        <v>5235</v>
+        <v>5232</v>
       </c>
       <c r="Q640">
-        <v>14453</v>
+        <v>14455</v>
       </c>
       <c r="R640">
         <v>397990</v>
@@ -34394,10 +34394,10 @@
         <v>1445142</v>
       </c>
       <c r="P641">
-        <v>5251</v>
+        <v>5252</v>
       </c>
       <c r="Q641">
-        <v>14478</v>
+        <v>14486</v>
       </c>
       <c r="R641">
         <v>405401</v>
@@ -34450,10 +34450,10 @@
         <v>1475491</v>
       </c>
       <c r="P642">
-        <v>5272</v>
+        <v>5278</v>
       </c>
       <c r="Q642">
-        <v>14509</v>
+        <v>14529</v>
       </c>
       <c r="R642">
         <v>417406</v>
@@ -34506,10 +34506,10 @@
         <v>1504895</v>
       </c>
       <c r="P643">
-        <v>5294</v>
+        <v>5295</v>
       </c>
       <c r="Q643">
-        <v>14565</v>
+        <v>14572</v>
       </c>
       <c r="R643">
         <v>423949</v>
@@ -34562,10 +34562,10 @@
         <v>1556926</v>
       </c>
       <c r="P644">
-        <v>5303</v>
+        <v>5298</v>
       </c>
       <c r="Q644">
-        <v>14589</v>
+        <v>14609</v>
       </c>
       <c r="R644">
         <v>422871</v>
@@ -34618,10 +34618,10 @@
         <v>1594529</v>
       </c>
       <c r="P645">
-        <v>5324</v>
+        <v>5320</v>
       </c>
       <c r="Q645">
-        <v>14603</v>
+        <v>14641</v>
       </c>
       <c r="R645">
         <v>428148</v>
@@ -34677,7 +34677,7 @@
         <v>5337</v>
       </c>
       <c r="Q646">
-        <v>14653</v>
+        <v>14660</v>
       </c>
       <c r="R646">
         <v>436947</v>
@@ -34730,10 +34730,10 @@
         <v>1688430</v>
       </c>
       <c r="P647">
-        <v>5359</v>
+        <v>5361</v>
       </c>
       <c r="Q647">
-        <v>14693</v>
+        <v>14676</v>
       </c>
       <c r="R647">
         <v>444351</v>
@@ -34786,10 +34786,10 @@
         <v>1727451</v>
       </c>
       <c r="P648">
-        <v>5366</v>
+        <v>5363</v>
       </c>
       <c r="Q648">
-        <v>14728</v>
+        <v>14713</v>
       </c>
       <c r="R648">
         <v>453531</v>
@@ -34842,10 +34842,10 @@
         <v>1772185</v>
       </c>
       <c r="P649">
-        <v>5378</v>
+        <v>5372</v>
       </c>
       <c r="Q649">
-        <v>14763</v>
+        <v>14755</v>
       </c>
       <c r="R649">
         <v>456086</v>
@@ -34898,10 +34898,10 @@
         <v>1816373</v>
       </c>
       <c r="P650">
-        <v>5390</v>
+        <v>5388</v>
       </c>
       <c r="Q650">
-        <v>14786</v>
+        <v>14781</v>
       </c>
       <c r="R650">
         <v>449421</v>
@@ -34954,10 +34954,10 @@
         <v>1855195</v>
       </c>
       <c r="P651">
-        <v>5404</v>
+        <v>5405</v>
       </c>
       <c r="Q651">
-        <v>14835</v>
+        <v>14826</v>
       </c>
       <c r="R651">
         <v>460527</v>
@@ -35010,10 +35010,10 @@
         <v>1888538</v>
       </c>
       <c r="P652">
-        <v>5414</v>
+        <v>5413</v>
       </c>
       <c r="Q652">
-        <v>14890</v>
+        <v>14894</v>
       </c>
       <c r="R652">
         <v>455814</v>
@@ -35066,10 +35066,10 @@
         <v>1925423</v>
       </c>
       <c r="P653">
-        <v>5418</v>
+        <v>5421</v>
       </c>
       <c r="Q653">
-        <v>14877</v>
+        <v>14884</v>
       </c>
       <c r="R653">
         <v>460896</v>
@@ -35125,7 +35125,7 @@
         <v>5420</v>
       </c>
       <c r="Q654">
-        <v>14905</v>
+        <v>14909</v>
       </c>
       <c r="R654">
         <v>458902</v>
@@ -35178,10 +35178,10 @@
         <v>1962179</v>
       </c>
       <c r="P655">
-        <v>5429</v>
+        <v>5423</v>
       </c>
       <c r="Q655">
-        <v>14915</v>
+        <v>14911</v>
       </c>
       <c r="R655">
         <v>454153</v>
@@ -35234,10 +35234,10 @@
         <v>1978635</v>
       </c>
       <c r="P656">
-        <v>5444</v>
+        <v>5443</v>
       </c>
       <c r="Q656">
-        <v>14946</v>
+        <v>14950</v>
       </c>
       <c r="R656">
         <v>464102</v>
@@ -35290,10 +35290,10 @@
         <v>1987043</v>
       </c>
       <c r="P657">
-        <v>5453</v>
+        <v>5468</v>
       </c>
       <c r="Q657">
-        <v>14973</v>
+        <v>14957</v>
       </c>
       <c r="R657">
         <v>469078</v>
@@ -35346,10 +35346,10 @@
         <v>2015413</v>
       </c>
       <c r="P658">
-        <v>5468</v>
+        <v>5479</v>
       </c>
       <c r="Q658">
-        <v>14986</v>
+        <v>14958</v>
       </c>
       <c r="R658">
         <v>470037</v>
@@ -35402,10 +35402,10 @@
         <v>2010974</v>
       </c>
       <c r="P659">
-        <v>5484</v>
+        <v>5492</v>
       </c>
       <c r="Q659">
-        <v>15012</v>
+        <v>14981</v>
       </c>
       <c r="R659">
         <v>474646</v>
@@ -35458,10 +35458,10 @@
         <v>2015374</v>
       </c>
       <c r="P660">
-        <v>5493</v>
+        <v>5502</v>
       </c>
       <c r="Q660">
-        <v>15022</v>
+        <v>14993</v>
       </c>
       <c r="R660">
         <v>472134</v>
@@ -35514,10 +35514,10 @@
         <v>2050568</v>
       </c>
       <c r="P661">
-        <v>5512</v>
+        <v>5515</v>
       </c>
       <c r="Q661">
-        <v>15036</v>
+        <v>15005</v>
       </c>
       <c r="R661">
         <v>466925</v>
@@ -35570,10 +35570,10 @@
         <v>2047434</v>
       </c>
       <c r="P662">
-        <v>5524</v>
+        <v>5525</v>
       </c>
       <c r="Q662">
-        <v>15053</v>
+        <v>15022</v>
       </c>
       <c r="R662">
         <v>468212</v>
@@ -35626,10 +35626,10 @@
         <v>2055482</v>
       </c>
       <c r="P663">
-        <v>5514</v>
+        <v>5525</v>
       </c>
       <c r="Q663">
-        <v>15071</v>
+        <v>15037</v>
       </c>
       <c r="R663">
         <v>467885</v>
@@ -35682,10 +35682,10 @@
         <v>2080486</v>
       </c>
       <c r="P664">
-        <v>5515</v>
+        <v>5523</v>
       </c>
       <c r="Q664">
-        <v>15087</v>
+        <v>15048</v>
       </c>
       <c r="R664">
         <v>470613</v>
@@ -35738,10 +35738,10 @@
         <v>2084190</v>
       </c>
       <c r="P665">
-        <v>5526</v>
+        <v>5522</v>
       </c>
       <c r="Q665">
-        <v>15114</v>
+        <v>15070</v>
       </c>
       <c r="R665">
         <v>475304</v>
@@ -35797,7 +35797,7 @@
         <v>5515</v>
       </c>
       <c r="Q666">
-        <v>15101</v>
+        <v>15094</v>
       </c>
       <c r="R666">
         <v>475285</v>
@@ -35850,10 +35850,10 @@
         <v>2109153</v>
       </c>
       <c r="P667">
-        <v>5511</v>
+        <v>5516</v>
       </c>
       <c r="Q667">
-        <v>15128</v>
+        <v>15126</v>
       </c>
       <c r="R667">
         <v>477452</v>
@@ -35906,10 +35906,10 @@
         <v>2109597</v>
       </c>
       <c r="P668">
-        <v>5505</v>
+        <v>5504</v>
       </c>
       <c r="Q668">
-        <v>15158</v>
+        <v>15146</v>
       </c>
       <c r="R668">
         <v>480190</v>
@@ -35962,10 +35962,10 @@
         <v>2122842</v>
       </c>
       <c r="P669">
-        <v>5478</v>
+        <v>5487</v>
       </c>
       <c r="Q669">
-        <v>15168</v>
+        <v>15132</v>
       </c>
       <c r="R669">
         <v>481748</v>
@@ -36018,10 +36018,10 @@
         <v>2132198</v>
       </c>
       <c r="P670">
-        <v>5486</v>
+        <v>5497</v>
       </c>
       <c r="Q670">
-        <v>15168</v>
+        <v>15132</v>
       </c>
       <c r="R670">
         <v>485022</v>
@@ -36032,7 +36032,7 @@
         <v>45961</v>
       </c>
       <c r="B671">
-        <v>924251</v>
+        <v>923951</v>
       </c>
       <c r="C671">
         <v>1689.4</v>
@@ -36044,7 +36044,7 @@
         <v>170539</v>
       </c>
       <c r="F671">
-        <v>6982033</v>
+        <v>6981949</v>
       </c>
       <c r="G671">
         <v>5980413</v>
@@ -36074,10 +36074,10 @@
         <v>2137467</v>
       </c>
       <c r="P671">
-        <v>5473</v>
+        <v>5493</v>
       </c>
       <c r="Q671">
-        <v>15186</v>
+        <v>15149</v>
       </c>
       <c r="R671">
         <v>486256</v>
@@ -36088,49 +36088,52 @@
         <v>45991</v>
       </c>
       <c r="B672">
-        <v>932682</v>
+        <v>944804</v>
+      </c>
+      <c r="C672">
+        <v>1766.7</v>
       </c>
       <c r="D672">
-        <v>380214</v>
+        <v>382977</v>
       </c>
       <c r="E672">
-        <v>169893</v>
+        <v>169583</v>
       </c>
       <c r="F672">
-        <v>7525804</v>
+        <v>7596783</v>
       </c>
       <c r="G672">
-        <v>5950591</v>
+        <v>5961933</v>
       </c>
       <c r="H672">
-        <v>2832070</v>
+        <v>2835263</v>
       </c>
       <c r="I672">
-        <v>487.68</v>
+        <v>487.66</v>
       </c>
       <c r="J672">
-        <v>40.09</v>
+        <v>40.08</v>
       </c>
       <c r="K672">
-        <v>15.52</v>
+        <v>15.51</v>
       </c>
       <c r="L672">
         <v>467.98</v>
       </c>
       <c r="M672">
-        <v>38587521</v>
+        <v>38590714</v>
       </c>
       <c r="N672">
-        <v>5422976</v>
+        <v>5425739</v>
       </c>
       <c r="O672">
-        <v>2151861</v>
+        <v>2151551</v>
       </c>
       <c r="P672">
-        <v>5474</v>
+        <v>5481</v>
       </c>
       <c r="Q672">
-        <v>15188</v>
+        <v>15145</v>
       </c>
     </row>
     <row r="673">
@@ -36138,49 +36141,63 @@
         <v>46022</v>
       </c>
       <c r="B673">
-        <v>1090401</v>
+        <v>1285497</v>
+      </c>
+      <c r="C673">
+        <v>1974.9</v>
       </c>
       <c r="D673">
-        <v>461712</v>
+        <v>547548</v>
       </c>
       <c r="E673">
-        <v>162551</v>
+        <v>192436</v>
       </c>
       <c r="F673">
-        <v>7294960</v>
+        <v>8746904</v>
       </c>
       <c r="G673">
-        <v>6474054</v>
+        <v>7817564</v>
       </c>
       <c r="H673">
-        <v>3033390</v>
+        <v>3794240</v>
       </c>
       <c r="I673">
-        <v>479.1</v>
+        <v>497.52</v>
       </c>
       <c r="J673">
-        <v>39.11</v>
+        <v>39.66</v>
       </c>
       <c r="K673">
         <v>15.51</v>
       </c>
       <c r="L673">
-        <v>469.22</v>
+        <v>471.08</v>
       </c>
       <c r="M673">
-        <v>38107671</v>
+        <v>38871714</v>
       </c>
       <c r="N673">
-        <v>5342825</v>
+        <v>5431424</v>
       </c>
       <c r="O673">
-        <v>2119925</v>
+        <v>2149500</v>
       </c>
       <c r="P673">
-        <v>5467</v>
+        <v>5471</v>
       </c>
       <c r="Q673">
-        <v>15206</v>
+        <v>15152</v>
+      </c>
+    </row>
+    <row r="674">
+      <c r="A674" s="2">
+        <v>46053</v>
+      </c>
+      <c r="P674">
+        <v>5453</v>
+      </c>
+      <c r="Q674">
+        <v>15162</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fim run (march 13)
</commit_message>
<xml_diff>
--- a/data/monthly_state_ui.xlsx
+++ b/data/monthly_state_ui.xlsx
@@ -355,7 +355,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:R674"/>
+  <dimension ref="A1:R675"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="20.7109375" style="2" customWidth="1"/>
@@ -36024,7 +36024,7 @@
         <v>15132</v>
       </c>
       <c r="R670">
-        <v>485022</v>
+        <v>487347</v>
       </c>
     </row>
     <row r="671">
@@ -36080,7 +36080,7 @@
         <v>15149</v>
       </c>
       <c r="R671">
-        <v>486256</v>
+        <v>487527</v>
       </c>
     </row>
     <row r="672">
@@ -36135,34 +36135,37 @@
       <c r="Q672">
         <v>15145</v>
       </c>
+      <c r="R672">
+        <v>486489</v>
+      </c>
     </row>
     <row r="673">
       <c r="A673" s="2">
         <v>46022</v>
       </c>
       <c r="B673">
-        <v>1285497</v>
+        <v>1285782</v>
       </c>
       <c r="C673">
         <v>1974.9</v>
       </c>
       <c r="D673">
-        <v>547548</v>
+        <v>547322</v>
       </c>
       <c r="E673">
-        <v>192436</v>
+        <v>192399</v>
       </c>
       <c r="F673">
-        <v>8746904</v>
+        <v>8741250</v>
       </c>
       <c r="G673">
-        <v>7817564</v>
+        <v>7813783</v>
       </c>
       <c r="H673">
-        <v>3794240</v>
+        <v>3792657</v>
       </c>
       <c r="I673">
-        <v>497.52</v>
+        <v>497.56</v>
       </c>
       <c r="J673">
         <v>39.66</v>
@@ -36174,30 +36177,86 @@
         <v>471.08</v>
       </c>
       <c r="M673">
-        <v>38871714</v>
+        <v>38870131</v>
       </c>
       <c r="N673">
-        <v>5431424</v>
+        <v>5431198</v>
       </c>
       <c r="O673">
-        <v>2149500</v>
+        <v>2149463</v>
       </c>
       <c r="P673">
-        <v>5471</v>
+        <v>5476</v>
       </c>
       <c r="Q673">
-        <v>15152</v>
+        <v>15151</v>
+      </c>
+      <c r="R673">
+        <v>483260</v>
       </c>
     </row>
     <row r="674">
       <c r="A674" s="2">
         <v>46053</v>
       </c>
+      <c r="B674">
+        <v>1161791</v>
+      </c>
+      <c r="C674">
+        <v>2105.6</v>
+      </c>
+      <c r="D674">
+        <v>642376</v>
+      </c>
+      <c r="E674">
+        <v>182859</v>
+      </c>
+      <c r="F674">
+        <v>8970205</v>
+      </c>
+      <c r="G674">
+        <v>7708449</v>
+      </c>
+      <c r="H674">
+        <v>3752803</v>
+      </c>
+      <c r="I674">
+        <v>498.09</v>
+      </c>
+      <c r="J674">
+        <v>39.77</v>
+      </c>
+      <c r="K674">
+        <v>15.61</v>
+      </c>
+      <c r="L674">
+        <v>473.72</v>
+      </c>
+      <c r="M674">
+        <v>38969876</v>
+      </c>
+      <c r="N674">
+        <v>5384517</v>
+      </c>
+      <c r="O674">
+        <v>2150953</v>
+      </c>
       <c r="P674">
-        <v>5453</v>
+        <v>5475</v>
       </c>
       <c r="Q674">
-        <v>15162</v>
+        <v>15161</v>
+      </c>
+    </row>
+    <row r="675">
+      <c r="A675" s="2">
+        <v>46081</v>
+      </c>
+      <c r="P675">
+        <v>5480</v>
+      </c>
+      <c r="Q675">
+        <v>15160</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
haver pull quarterly updates
</commit_message>
<xml_diff>
--- a/data/monthly_state_ui.xlsx
+++ b/data/monthly_state_ui.xlsx
@@ -9869,7 +9869,7 @@
         <v>235008</v>
       </c>
       <c r="F194">
-        <v>14582389</v>
+        <v>14713714</v>
       </c>
       <c r="G194">
         <v>13027499</v>
@@ -9975,7 +9975,7 @@
         <v>219934</v>
       </c>
       <c r="F196">
-        <v>12935633</v>
+        <v>13070015</v>
       </c>
       <c r="G196">
         <v>11730221</v>
@@ -10134,7 +10134,7 @@
         <v>212380</v>
       </c>
       <c r="F199">
-        <v>10143793</v>
+        <v>10180428</v>
       </c>
       <c r="G199">
         <v>9028611</v>
@@ -10293,7 +10293,7 @@
         <v>211859</v>
       </c>
       <c r="F202">
-        <v>9577738</v>
+        <v>10031217</v>
       </c>
       <c r="G202">
         <v>8724780</v>
@@ -10346,7 +10346,7 @@
         <v>223173</v>
       </c>
       <c r="F203">
-        <v>9570267</v>
+        <v>9819412</v>
       </c>
       <c r="G203">
         <v>8695175</v>
@@ -35528,28 +35528,28 @@
         <v>45688</v>
       </c>
       <c r="B662">
-        <v>1229039</v>
+        <v>1229141</v>
       </c>
       <c r="C662">
         <v>2144.7</v>
       </c>
       <c r="D662">
-        <v>689057</v>
+        <v>688712</v>
       </c>
       <c r="E662">
-        <v>181369</v>
+        <v>181496</v>
       </c>
       <c r="F662">
-        <v>9270872</v>
+        <v>9270989</v>
       </c>
       <c r="G662">
-        <v>7923862</v>
+        <v>7926461</v>
       </c>
       <c r="H662">
-        <v>3653058</v>
+        <v>3653758</v>
       </c>
       <c r="I662">
-        <v>469.31</v>
+        <v>469.22</v>
       </c>
       <c r="J662">
         <v>38.94</v>
@@ -35558,16 +35558,16 @@
         <v>15.17</v>
       </c>
       <c r="L662">
-        <v>454.83</v>
+        <v>454.82</v>
       </c>
       <c r="M662">
-        <v>36187127</v>
+        <v>36187827</v>
       </c>
       <c r="N662">
-        <v>5341606</v>
+        <v>5341261</v>
       </c>
       <c r="O662">
-        <v>2047434</v>
+        <v>2047561</v>
       </c>
       <c r="P662">
         <v>5525</v>
@@ -35584,28 +35584,28 @@
         <v>45716</v>
       </c>
       <c r="B663">
-        <v>903834</v>
+        <v>903900</v>
       </c>
       <c r="C663">
         <v>2141</v>
       </c>
       <c r="D663">
-        <v>483723</v>
+        <v>483300</v>
       </c>
       <c r="E663">
-        <v>165517</v>
+        <v>165518</v>
       </c>
       <c r="F663">
-        <v>8657553</v>
+        <v>8657657</v>
       </c>
       <c r="G663">
-        <v>7509946</v>
+        <v>7509945</v>
       </c>
       <c r="H663">
-        <v>3480178</v>
+        <v>3480197</v>
       </c>
       <c r="I663">
-        <v>471.52</v>
+        <v>471.51</v>
       </c>
       <c r="J663">
         <v>39.22</v>
@@ -35614,16 +35614,16 @@
         <v>15.21</v>
       </c>
       <c r="L663">
-        <v>455.94</v>
+        <v>455.93</v>
       </c>
       <c r="M663">
-        <v>36328230</v>
+        <v>36328948</v>
       </c>
       <c r="N663">
-        <v>5334772</v>
+        <v>5334004</v>
       </c>
       <c r="O663">
-        <v>2055482</v>
+        <v>2055610</v>
       </c>
       <c r="P663">
         <v>5525</v>
@@ -35640,46 +35640,46 @@
         <v>45747</v>
       </c>
       <c r="B664">
-        <v>889619</v>
+        <v>889680</v>
       </c>
       <c r="C664">
         <v>2065.1</v>
       </c>
       <c r="D664">
-        <v>431634</v>
+        <v>431167</v>
       </c>
       <c r="E664">
-        <v>188778</v>
+        <v>188784</v>
       </c>
       <c r="F664">
-        <v>9621688</v>
+        <v>9621785</v>
       </c>
       <c r="G664">
-        <v>8149650</v>
+        <v>8149709</v>
       </c>
       <c r="H664">
-        <v>3743494</v>
+        <v>3743539</v>
       </c>
       <c r="I664">
-        <v>467.76</v>
+        <v>467.75</v>
       </c>
       <c r="J664">
-        <v>39.58</v>
+        <v>39.59</v>
       </c>
       <c r="K664">
         <v>15.3</v>
       </c>
       <c r="L664">
-        <v>457.11</v>
+        <v>457.1</v>
       </c>
       <c r="M664">
-        <v>36783747</v>
+        <v>36784511</v>
       </c>
       <c r="N664">
-        <v>5357347</v>
+        <v>5356112</v>
       </c>
       <c r="O664">
-        <v>2080486</v>
+        <v>2080620</v>
       </c>
       <c r="P664">
         <v>5523</v>
@@ -35696,46 +35696,46 @@
         <v>45777</v>
       </c>
       <c r="B665">
-        <v>942921</v>
+        <v>942976</v>
       </c>
       <c r="C665">
         <v>1877</v>
       </c>
       <c r="D665">
-        <v>401308</v>
+        <v>400726</v>
       </c>
       <c r="E665">
-        <v>189319</v>
+        <v>189309</v>
       </c>
       <c r="F665">
-        <v>7912994</v>
+        <v>7913076</v>
       </c>
       <c r="G665">
-        <v>6972902</v>
+        <v>6972826</v>
       </c>
       <c r="H665">
-        <v>3204874</v>
+        <v>3204868</v>
       </c>
       <c r="I665">
-        <v>468.53</v>
+        <v>468.52</v>
       </c>
       <c r="J665">
         <v>39.47</v>
       </c>
       <c r="K665">
-        <v>15.22</v>
+        <v>15.23</v>
       </c>
       <c r="L665">
-        <v>458.19</v>
+        <v>458.18</v>
       </c>
       <c r="M665">
-        <v>36811988</v>
+        <v>36812745</v>
       </c>
       <c r="N665">
-        <v>5375518</v>
+        <v>5373701</v>
       </c>
       <c r="O665">
-        <v>2084190</v>
+        <v>2084314</v>
       </c>
       <c r="P665">
         <v>5522</v>
@@ -35752,46 +35752,46 @@
         <v>45808</v>
       </c>
       <c r="B666">
-        <v>894785</v>
+        <v>894858</v>
       </c>
       <c r="C666">
         <v>1760.6</v>
       </c>
       <c r="D666">
-        <v>371539</v>
+        <v>370965</v>
       </c>
       <c r="E666">
-        <v>174208</v>
+        <v>174214</v>
       </c>
       <c r="F666">
-        <v>7224983</v>
+        <v>7225163</v>
       </c>
       <c r="G666">
-        <v>6139864</v>
+        <v>6140058</v>
       </c>
       <c r="H666">
-        <v>2798144</v>
+        <v>2798186</v>
       </c>
       <c r="I666">
-        <v>465.28</v>
+        <v>465.25</v>
       </c>
       <c r="J666">
         <v>39.76</v>
       </c>
       <c r="K666">
-        <v>15.27</v>
+        <v>15.28</v>
       </c>
       <c r="L666">
-        <v>458.9</v>
+        <v>458.88</v>
       </c>
       <c r="M666">
-        <v>36916392</v>
+        <v>36917191</v>
       </c>
       <c r="N666">
-        <v>5368085</v>
+        <v>5365694</v>
       </c>
       <c r="O666">
-        <v>2089888</v>
+        <v>2090018</v>
       </c>
       <c r="P666">
         <v>5515</v>
@@ -35808,28 +35808,28 @@
         <v>45838</v>
       </c>
       <c r="B667">
-        <v>1031839</v>
+        <v>1031918</v>
       </c>
       <c r="C667">
         <v>1860.9</v>
       </c>
       <c r="D667">
-        <v>457394</v>
+        <v>456816</v>
       </c>
       <c r="E667">
-        <v>178819</v>
+        <v>178825</v>
       </c>
       <c r="F667">
-        <v>8573274</v>
+        <v>8573406</v>
       </c>
       <c r="G667">
-        <v>6954166</v>
+        <v>6954221</v>
       </c>
       <c r="H667">
-        <v>3100962</v>
+        <v>3100995</v>
       </c>
       <c r="I667">
-        <v>455.27</v>
+        <v>455.28</v>
       </c>
       <c r="J667">
         <v>39.55</v>
@@ -35838,16 +35838,16 @@
         <v>15.3</v>
       </c>
       <c r="L667">
-        <v>459.67</v>
+        <v>459.66</v>
       </c>
       <c r="M667">
-        <v>37393949</v>
+        <v>37394781</v>
       </c>
       <c r="N667">
-        <v>5419922</v>
+        <v>5416953</v>
       </c>
       <c r="O667">
-        <v>2109153</v>
+        <v>2109289</v>
       </c>
       <c r="P667">
         <v>5516</v>
@@ -35864,46 +35864,46 @@
         <v>45869</v>
       </c>
       <c r="B668">
-        <v>981550</v>
+        <v>981627</v>
       </c>
       <c r="C668">
         <v>2004.2</v>
       </c>
       <c r="D668">
-        <v>510167</v>
+        <v>509550</v>
       </c>
       <c r="E668">
-        <v>182275</v>
+        <v>182609</v>
       </c>
       <c r="F668">
-        <v>8421915</v>
+        <v>8421960</v>
       </c>
       <c r="G668">
-        <v>7295233</v>
+        <v>7300670</v>
       </c>
       <c r="H668">
-        <v>3288759</v>
+        <v>3290187</v>
       </c>
       <c r="I668">
-        <v>459.83</v>
+        <v>459.66</v>
       </c>
       <c r="J668">
-        <v>39.49</v>
+        <v>39.51</v>
       </c>
       <c r="K668">
-        <v>15.32</v>
+        <v>15.33</v>
       </c>
       <c r="L668">
-        <v>461.59</v>
+        <v>461.56</v>
       </c>
       <c r="M668">
-        <v>37517883</v>
+        <v>37520143</v>
       </c>
       <c r="N668">
-        <v>5407963</v>
+        <v>5404377</v>
       </c>
       <c r="O668">
-        <v>2109598</v>
+        <v>2110068</v>
       </c>
       <c r="P668">
         <v>5504</v>
@@ -35920,46 +35920,46 @@
         <v>45900</v>
       </c>
       <c r="B669">
-        <v>837631</v>
+        <v>837602</v>
       </c>
       <c r="C669">
         <v>1906.9</v>
       </c>
       <c r="D669">
-        <v>406108</v>
+        <v>405660</v>
       </c>
       <c r="E669">
-        <v>177776</v>
+        <v>177777</v>
       </c>
       <c r="F669">
-        <v>8429756</v>
+        <v>8429794</v>
       </c>
       <c r="G669">
-        <v>6919792</v>
+        <v>6919811</v>
       </c>
       <c r="H669">
-        <v>3096034</v>
+        <v>3096051</v>
       </c>
       <c r="I669">
-        <v>457.06</v>
+        <v>457.05</v>
       </c>
       <c r="J669">
-        <v>39.79</v>
+        <v>39.81</v>
       </c>
       <c r="K669">
-        <v>15.41</v>
+        <v>15.42</v>
       </c>
       <c r="L669">
-        <v>462.81</v>
+        <v>462.78</v>
       </c>
       <c r="M669">
-        <v>37812985</v>
+        <v>37815262</v>
       </c>
       <c r="N669">
-        <v>5405470</v>
+        <v>5401436</v>
       </c>
       <c r="O669">
-        <v>2122844</v>
+        <v>2123315</v>
       </c>
       <c r="P669">
         <v>5487</v>
@@ -35976,46 +35976,46 @@
         <v>45930</v>
       </c>
       <c r="B670">
-        <v>852802</v>
+        <v>852782</v>
       </c>
       <c r="C670">
         <v>1709.7</v>
       </c>
       <c r="D670">
-        <v>369998</v>
+        <v>369609</v>
       </c>
       <c r="E670">
         <v>178887</v>
       </c>
       <c r="F670">
-        <v>7502522</v>
+        <v>7502566</v>
       </c>
       <c r="G670">
-        <v>6623344</v>
+        <v>6623253</v>
       </c>
       <c r="H670">
-        <v>3039165</v>
+        <v>3039174</v>
       </c>
       <c r="I670">
         <v>469.54</v>
       </c>
       <c r="J670">
-        <v>39.8</v>
+        <v>39.82</v>
       </c>
       <c r="K670">
-        <v>15.43</v>
+        <v>15.44</v>
       </c>
       <c r="L670">
-        <v>464.21</v>
+        <v>464.18</v>
       </c>
       <c r="M670">
-        <v>38098604</v>
+        <v>38100889</v>
       </c>
       <c r="N670">
-        <v>5424200</v>
+        <v>5419777</v>
       </c>
       <c r="O670">
-        <v>2132204</v>
+        <v>2132675</v>
       </c>
       <c r="P670">
         <v>5497</v>
@@ -36032,46 +36032,46 @@
         <v>45961</v>
       </c>
       <c r="B671">
-        <v>923951</v>
+        <v>923962</v>
       </c>
       <c r="C671">
         <v>1689.4</v>
       </c>
       <c r="D671">
-        <v>380062</v>
+        <v>379561</v>
       </c>
       <c r="E671">
-        <v>170539</v>
+        <v>170537</v>
       </c>
       <c r="F671">
-        <v>6981949</v>
+        <v>6981993</v>
       </c>
       <c r="G671">
-        <v>5980413</v>
+        <v>5980353</v>
       </c>
       <c r="H671">
-        <v>2837711</v>
+        <v>2837717</v>
       </c>
       <c r="I671">
-        <v>485.72</v>
+        <v>485.7</v>
       </c>
       <c r="J671">
-        <v>39.76</v>
+        <v>39.79</v>
       </c>
       <c r="K671">
-        <v>15.48</v>
+        <v>15.49</v>
       </c>
       <c r="L671">
-        <v>466.12</v>
+        <v>466.09</v>
       </c>
       <c r="M671">
-        <v>38269280</v>
+        <v>38271571</v>
       </c>
       <c r="N671">
-        <v>5411752</v>
+        <v>5406828</v>
       </c>
       <c r="O671">
-        <v>2137473</v>
+        <v>2137942</v>
       </c>
       <c r="P671">
         <v>5493</v>
@@ -36088,46 +36088,46 @@
         <v>45991</v>
       </c>
       <c r="B672">
-        <v>945078</v>
+        <v>945075</v>
       </c>
       <c r="C672">
         <v>1766.7</v>
       </c>
       <c r="D672">
-        <v>382977</v>
+        <v>382611</v>
       </c>
       <c r="E672">
-        <v>169583</v>
+        <v>169582</v>
       </c>
       <c r="F672">
-        <v>7596783</v>
+        <v>7596869</v>
       </c>
       <c r="G672">
-        <v>5961933</v>
+        <v>5961957</v>
       </c>
       <c r="H672">
-        <v>2835263</v>
+        <v>2835269</v>
       </c>
       <c r="I672">
-        <v>487.66</v>
+        <v>487.64</v>
       </c>
       <c r="J672">
-        <v>40.08</v>
+        <v>40.11</v>
       </c>
       <c r="K672">
-        <v>15.51</v>
+        <v>15.53</v>
       </c>
       <c r="L672">
-        <v>467.98</v>
+        <v>467.95</v>
       </c>
       <c r="M672">
-        <v>38590883</v>
+        <v>38593180</v>
       </c>
       <c r="N672">
-        <v>5425830</v>
+        <v>5420540</v>
       </c>
       <c r="O672">
-        <v>2151557</v>
+        <v>2152025</v>
       </c>
       <c r="P672">
         <v>5481</v>
@@ -36144,46 +36144,46 @@
         <v>46022</v>
       </c>
       <c r="B673">
-        <v>1285782</v>
+        <v>1285761</v>
       </c>
       <c r="C673">
         <v>1974.9</v>
       </c>
       <c r="D673">
-        <v>547322</v>
+        <v>546902</v>
       </c>
       <c r="E673">
-        <v>192399</v>
+        <v>192398</v>
       </c>
       <c r="F673">
-        <v>8741250</v>
+        <v>8741358</v>
       </c>
       <c r="G673">
-        <v>7813783</v>
+        <v>7813813</v>
       </c>
       <c r="H673">
-        <v>3792657</v>
+        <v>3792659</v>
       </c>
       <c r="I673">
-        <v>497.56</v>
+        <v>497.54</v>
       </c>
       <c r="J673">
-        <v>39.66</v>
+        <v>39.69</v>
       </c>
       <c r="K673">
-        <v>15.51</v>
+        <v>15.53</v>
       </c>
       <c r="L673">
-        <v>471.08</v>
+        <v>471.05</v>
       </c>
       <c r="M673">
-        <v>38870300</v>
+        <v>38872600</v>
       </c>
       <c r="N673">
-        <v>5431289</v>
+        <v>5425579</v>
       </c>
       <c r="O673">
-        <v>2149469</v>
+        <v>2149936</v>
       </c>
       <c r="P673">
         <v>5476</v>
@@ -36200,46 +36200,46 @@
         <v>46053</v>
       </c>
       <c r="B674">
-        <v>1161466</v>
+        <v>1161429</v>
       </c>
       <c r="C674">
         <v>2105.6</v>
       </c>
       <c r="D674">
-        <v>642221</v>
+        <v>641813</v>
       </c>
       <c r="E674">
-        <v>182707</v>
+        <v>182706</v>
       </c>
       <c r="F674">
-        <v>8967994</v>
+        <v>9000893</v>
       </c>
       <c r="G674">
-        <v>7706482</v>
+        <v>7706483</v>
       </c>
       <c r="H674">
         <v>3752090</v>
       </c>
       <c r="I674">
-        <v>498.12</v>
+        <v>498.11</v>
       </c>
       <c r="J674">
-        <v>39.77</v>
+        <v>39.8</v>
       </c>
       <c r="K674">
-        <v>15.61</v>
+        <v>15.62</v>
       </c>
       <c r="L674">
-        <v>473.73</v>
+        <v>473.7</v>
       </c>
       <c r="M674">
-        <v>38969333</v>
+        <v>38970932</v>
       </c>
       <c r="N674">
-        <v>5384453</v>
+        <v>5378680</v>
       </c>
       <c r="O674">
-        <v>2150807</v>
+        <v>2151146</v>
       </c>
       <c r="P674">
         <v>5479</v>
@@ -36256,43 +36256,46 @@
         <v>46081</v>
       </c>
       <c r="B675">
-        <v>870690</v>
+        <v>870653</v>
+      </c>
+      <c r="C675">
+        <v>2112.7</v>
       </c>
       <c r="D675">
-        <v>501489</v>
+        <v>500950</v>
       </c>
       <c r="E675">
         <v>166604</v>
       </c>
       <c r="F675">
-        <v>8658844</v>
+        <v>8658902</v>
       </c>
       <c r="G675">
-        <v>7497492</v>
+        <v>7497563</v>
       </c>
       <c r="H675">
-        <v>3707842</v>
+        <v>3707864</v>
       </c>
       <c r="I675">
-        <v>505.41</v>
+        <v>505.39</v>
       </c>
       <c r="J675">
-        <v>39.81</v>
+        <v>39.85</v>
       </c>
       <c r="K675">
-        <v>15.55</v>
+        <v>15.57</v>
       </c>
       <c r="L675">
-        <v>476.76</v>
+        <v>476.73</v>
       </c>
       <c r="M675">
-        <v>39196997</v>
+        <v>39198599</v>
       </c>
       <c r="N675">
-        <v>5402219</v>
+        <v>5396330</v>
       </c>
       <c r="O675">
-        <v>2151894</v>
+        <v>2152232</v>
       </c>
       <c r="P675">
         <v>5480</v>
@@ -36304,6 +36307,45 @@
     <row r="676">
       <c r="A676" s="2">
         <v>46112</v>
+      </c>
+      <c r="B676">
+        <v>865415</v>
+      </c>
+      <c r="D676">
+        <v>424816</v>
+      </c>
+      <c r="E676">
+        <v>193591</v>
+      </c>
+      <c r="F676">
+        <v>9678293</v>
+      </c>
+      <c r="G676">
+        <v>8464959</v>
+      </c>
+      <c r="H676">
+        <v>4181624</v>
+      </c>
+      <c r="I676">
+        <v>506.87</v>
+      </c>
+      <c r="J676">
+        <v>39.8</v>
+      </c>
+      <c r="K676">
+        <v>15.65</v>
+      </c>
+      <c r="L676">
+        <v>480.62</v>
+      </c>
+      <c r="M676">
+        <v>39636684</v>
+      </c>
+      <c r="N676">
+        <v>5389979</v>
+      </c>
+      <c r="O676">
+        <v>2157039</v>
       </c>
       <c r="P676">
         <v>5476</v>

</xml_diff>

<commit_message>
update to haver automation process to enclude SB
</commit_message>
<xml_diff>
--- a/data/monthly_state_ui.xlsx
+++ b/data/monthly_state_ui.xlsx
@@ -355,7 +355,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:R677"/>
+  <dimension ref="A1:R678"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="20.7109375" style="2" customWidth="1"/>
@@ -10770,7 +10770,7 @@
         <v>206268</v>
       </c>
       <c r="F211">
-        <v>9409396</v>
+        <v>9373396</v>
       </c>
       <c r="G211">
         <v>8264366</v>
@@ -10779,7 +10779,7 @@
         <v>1120652</v>
       </c>
       <c r="I211">
-        <v>140.32</v>
+        <v>140.12</v>
       </c>
       <c r="J211">
         <v>32.1</v>
@@ -36032,7 +36032,7 @@
         <v>45961</v>
       </c>
       <c r="B671">
-        <v>924286</v>
+        <v>924025</v>
       </c>
       <c r="C671">
         <v>1689.4</v>
@@ -36041,16 +36041,16 @@
         <v>379596</v>
       </c>
       <c r="E671">
-        <v>170538</v>
+        <v>170543</v>
       </c>
       <c r="F671">
-        <v>6982020</v>
+        <v>6979391</v>
       </c>
       <c r="G671">
-        <v>5980436</v>
+        <v>5980439</v>
       </c>
       <c r="H671">
-        <v>2837778</v>
+        <v>2837785</v>
       </c>
       <c r="I671">
         <v>485.7</v>
@@ -36065,13 +36065,13 @@
         <v>466.09</v>
       </c>
       <c r="M671">
-        <v>38270538</v>
+        <v>38270545</v>
       </c>
       <c r="N671">
         <v>5406862</v>
       </c>
       <c r="O671">
-        <v>2137944</v>
+        <v>2137949</v>
       </c>
       <c r="P671">
         <v>5493</v>
@@ -36088,7 +36088,7 @@
         <v>45991</v>
       </c>
       <c r="B672">
-        <v>945075</v>
+        <v>945119</v>
       </c>
       <c r="C672">
         <v>1766.7</v>
@@ -36097,13 +36097,13 @@
         <v>382611</v>
       </c>
       <c r="E672">
-        <v>169582</v>
+        <v>169586</v>
       </c>
       <c r="F672">
-        <v>7596869</v>
+        <v>7594932</v>
       </c>
       <c r="G672">
-        <v>5961957</v>
+        <v>5961960</v>
       </c>
       <c r="H672">
         <v>2835269</v>
@@ -36121,13 +36121,13 @@
         <v>467.95</v>
       </c>
       <c r="M672">
-        <v>38592147</v>
+        <v>38592155</v>
       </c>
       <c r="N672">
         <v>5420574</v>
       </c>
       <c r="O672">
-        <v>2152027</v>
+        <v>2152036</v>
       </c>
       <c r="P672">
         <v>5481</v>
@@ -36144,7 +36144,7 @@
         <v>46022</v>
       </c>
       <c r="B673">
-        <v>1286768</v>
+        <v>1286403</v>
       </c>
       <c r="C673">
         <v>1974.9</v>
@@ -36153,16 +36153,16 @@
         <v>546936</v>
       </c>
       <c r="E673">
-        <v>192398</v>
+        <v>192404</v>
       </c>
       <c r="F673">
-        <v>8744744</v>
+        <v>8732950</v>
       </c>
       <c r="G673">
-        <v>7813893</v>
+        <v>7813896</v>
       </c>
       <c r="H673">
-        <v>3792726</v>
+        <v>3792728</v>
       </c>
       <c r="I673">
         <v>497.55</v>
@@ -36177,13 +36177,13 @@
         <v>471.05</v>
       </c>
       <c r="M673">
-        <v>38871633</v>
+        <v>38871643</v>
       </c>
       <c r="N673">
         <v>5425647</v>
       </c>
       <c r="O673">
-        <v>2149938</v>
+        <v>2149953</v>
       </c>
       <c r="P673">
         <v>5476</v>
@@ -36200,7 +36200,7 @@
         <v>46053</v>
       </c>
       <c r="B674">
-        <v>1153389</v>
+        <v>1152536</v>
       </c>
       <c r="C674">
         <v>2105.6</v>
@@ -36209,16 +36209,16 @@
         <v>637251</v>
       </c>
       <c r="E674">
-        <v>180631</v>
+        <v>180638</v>
       </c>
       <c r="F674">
-        <v>8926453</v>
+        <v>8916656</v>
       </c>
       <c r="G674">
-        <v>7637362</v>
+        <v>7637367</v>
       </c>
       <c r="H674">
-        <v>3737121</v>
+        <v>3737129</v>
       </c>
       <c r="I674">
         <v>500.63</v>
@@ -36233,13 +36233,13 @@
         <v>473.91</v>
       </c>
       <c r="M674">
-        <v>38954996</v>
+        <v>38955015</v>
       </c>
       <c r="N674">
         <v>5374186</v>
       </c>
       <c r="O674">
-        <v>2149073</v>
+        <v>2149095</v>
       </c>
       <c r="P674">
         <v>5479</v>
@@ -36256,7 +36256,7 @@
         <v>46081</v>
       </c>
       <c r="B675">
-        <v>869941</v>
+        <v>869311</v>
       </c>
       <c r="C675">
         <v>2112.7</v>
@@ -36265,16 +36265,16 @@
         <v>500092</v>
       </c>
       <c r="E675">
-        <v>166300</v>
+        <v>166311</v>
       </c>
       <c r="F675">
-        <v>8670269</v>
+        <v>8661433</v>
       </c>
       <c r="G675">
         <v>7505641</v>
       </c>
       <c r="H675">
-        <v>3709920</v>
+        <v>3462193</v>
       </c>
       <c r="I675">
         <v>505.07</v>
@@ -36289,13 +36289,13 @@
         <v>476.92</v>
       </c>
       <c r="M675">
-        <v>39184719</v>
+        <v>38937011</v>
       </c>
       <c r="N675">
         <v>5390978</v>
       </c>
       <c r="O675">
-        <v>2149855</v>
+        <v>2149888</v>
       </c>
       <c r="P675">
         <v>5473</v>
@@ -36304,7 +36304,7 @@
         <v>15159</v>
       </c>
       <c r="R675">
-        <v>490094</v>
+        <v>491753</v>
       </c>
     </row>
     <row r="676">
@@ -36312,25 +36312,25 @@
         <v>46112</v>
       </c>
       <c r="B676">
-        <v>863458</v>
+        <v>862825</v>
       </c>
       <c r="C676">
         <v>2009.6</v>
       </c>
       <c r="D676">
-        <v>423395</v>
+        <v>423396</v>
       </c>
       <c r="E676">
-        <v>192720</v>
+        <v>192723</v>
       </c>
       <c r="F676">
-        <v>9700930</v>
+        <v>9689666</v>
       </c>
       <c r="G676">
-        <v>8462470</v>
+        <v>8462498</v>
       </c>
       <c r="H676">
-        <v>4169986</v>
+        <v>4170006</v>
       </c>
       <c r="I676">
         <v>503.96</v>
@@ -36345,33 +36345,89 @@
         <v>480.53</v>
       </c>
       <c r="M676">
-        <v>39611166</v>
+        <v>39363478</v>
       </c>
       <c r="N676">
-        <v>5383206</v>
+        <v>5383207</v>
       </c>
       <c r="O676">
-        <v>2153791</v>
+        <v>2153827</v>
       </c>
       <c r="P676">
-        <v>5471</v>
+        <v>5469</v>
       </c>
       <c r="Q676">
-        <v>15171</v>
+        <v>15182</v>
       </c>
       <c r="R676">
-        <v>489842</v>
+        <v>492834</v>
       </c>
     </row>
     <row r="677">
       <c r="A677" s="2">
         <v>46142</v>
       </c>
+      <c r="B677">
+        <v>850091</v>
+      </c>
+      <c r="C677">
+        <v>1750.1</v>
+      </c>
+      <c r="D677">
+        <v>358829</v>
+      </c>
+      <c r="E677">
+        <v>176044</v>
+      </c>
+      <c r="F677">
+        <v>7445078</v>
+      </c>
+      <c r="G677">
+        <v>6575681</v>
+      </c>
+      <c r="H677">
+        <v>3235588</v>
+      </c>
+      <c r="I677">
+        <v>504.74</v>
+      </c>
+      <c r="J677">
+        <v>39.59</v>
+      </c>
+      <c r="K677">
+        <v>15.7</v>
+      </c>
+      <c r="L677">
+        <v>483.42</v>
+      </c>
+      <c r="M677">
+        <v>39394198</v>
+      </c>
+      <c r="N677">
+        <v>5341310</v>
+      </c>
+      <c r="O677">
+        <v>2140562</v>
+      </c>
       <c r="P677">
-        <v>5472</v>
+        <v>5471</v>
       </c>
       <c r="Q677">
-        <v>15171</v>
+        <v>15188</v>
+      </c>
+      <c r="R677">
+        <v>493202</v>
+      </c>
+    </row>
+    <row r="678">
+      <c r="A678" s="2">
+        <v>46173</v>
+      </c>
+      <c r="P678">
+        <v>5467</v>
+      </c>
+      <c r="Q678">
+        <v>15243</v>
       </c>
     </row>
   </sheetData>

</xml_diff>